<commit_message>
Fix column-width pixel conversion formula
The (pixels-5)/7 formula used in the previous commit rendered every
column 5px narrower than intended (confirmed against on-screen
measurements: 100/59/220/135/135 vs targets 105/64/225/140/140).
Correct formula is pixels/7 with no offset: A=15.0, B=9.14, C=32.14,
D=20.0, E=20.0. Fixture regenerated to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/Example_2026_Invoice_07162026.xlsx
+++ b/tests/fixtures/Example_2026_Invoice_07162026.xlsx
@@ -619,11 +619,11 @@
   <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14.29" customWidth="1" min="1" max="1"/>
-    <col width="8.43" customWidth="1" min="2" max="2"/>
-    <col width="31.43" customWidth="1" min="3" max="3"/>
-    <col width="19.29" customWidth="1" min="4" max="4"/>
-    <col width="19.29" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="9.140000000000001" customWidth="1" min="2" max="2"/>
+    <col width="32.14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">

</xml_diff>